<commit_message>
Refactor: switch production counting to pieces per shift
</commit_message>
<xml_diff>
--- a/project/config/machine_config_file.xlsx
+++ b/project/config/machine_config_file.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jsochacki\Desktop\Python\Tkinter\production-counting\project\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{880E2158-2ABC-4E75-928D-7FA8DB3BCDEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30F646D1-F6ED-49D0-B85F-7446BBAA1F71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-195" windowWidth="29040" windowHeight="15720" xr2:uid="{7ECE9BE7-212F-406A-B24E-5B0CDEAB2EA7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7ECE9BE7-212F-406A-B24E-5B0CDEAB2EA7}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -41,15 +41,9 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
-    <t>machine</t>
-  </si>
-  <si>
     <t>speed_m_per_min</t>
   </si>
   <si>
-    <t>count_by_m</t>
-  </si>
-  <si>
     <t>WLO-U001</t>
   </si>
   <si>
@@ -90,6 +84,12 @@
   </si>
   <si>
     <t>WLO-U014</t>
+  </si>
+  <si>
+    <t>count_by_shift</t>
+  </si>
+  <si>
+    <t>workplace</t>
   </si>
 </sst>
 </file>
@@ -472,23 +472,23 @@
   <cols>
     <col min="1" max="1" width="12.140625" customWidth="1"/>
     <col min="2" max="2" width="19.28515625" customWidth="1"/>
-    <col min="3" max="3" width="13.28515625" customWidth="1"/>
+    <col min="3" max="3" width="15" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2">
         <v>14</v>
@@ -499,7 +499,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="B3">
         <v>8</v>
@@ -510,7 +510,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4">
         <v>12</v>
@@ -521,7 +521,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B5">
         <v>8</v>
@@ -532,7 +532,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B6">
         <v>10</v>
@@ -543,7 +543,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B7">
         <v>10</v>
@@ -554,7 +554,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B8">
         <v>8</v>
@@ -565,7 +565,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9">
         <v>0</v>
@@ -576,7 +576,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B10">
         <v>12</v>
@@ -587,7 +587,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B11">
         <v>14</v>
@@ -598,7 +598,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B12">
         <v>12</v>
@@ -609,7 +609,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B13">
         <v>12</v>
@@ -620,7 +620,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B14">
         <v>12</v>
@@ -631,7 +631,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B15">
         <v>14</v>

</xml_diff>